<commit_message>
add Week3 compare class diagram sequence diagram and activity diagram with AI
</commit_message>
<xml_diff>
--- a/AI Audit Log_TRanVanDong_DE180115.xlsx
+++ b/AI Audit Log_TRanVanDong_DE180115.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08818552-C800-4587-8B7F-9832C1D45D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB173833-B8FA-4B66-9B7C-E452AA80AFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week1" sheetId="1" r:id="rId1"/>
     <sheet name="Week2" sheetId="2" r:id="rId2"/>
-    <sheet name="Assignment 2" sheetId="3" r:id="rId3"/>
+    <sheet name="Week3" sheetId="3" r:id="rId3"/>
     <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="46">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -234,6 +234,76 @@
   </si>
   <si>
     <t xml:space="preserve">Làm Báo Cáo và tìm hiểu các sơ đồ trong bản báo cáo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiết kế Class Diagram và so sánh thiết kế của AI </t>
+  </si>
+  <si>
+    <t>"dựa vào hình ảnh classDiagram tôi vẽ cho bài 1 bạn hãy so sánh Class Diagram do tôi tự thiết kế với Class Diagram do bạn đề xuất cho hệ thống AutoGo car rental."</t>
+  </si>
+  <si>
+    <t>AI Response (tóm tắt):
+AI so sánh Class Diagram của em với phiên bản đề xuất, đánh giá 7.0 – 7.5/10. Điểm mạnh: đúng inheritance, Generic Repository. Điểm yếu: thiếu BookingService, mối quan hệ Booking-Vehicle chưa chuẩn, chưa thể hiện rõ dependency Service → Repository.
+Quyết định của người học: 
+Chỉnh sửa bằng cách: bổ sung BookingService, đổi Vehicle thành Car, sửa relationship Booking-Car thành Association, và thêm dependency. Sử dụng phiên bản chỉnh sửa để nộp bài.</t>
+  </si>
+  <si>
+    <t>AI Response (tóm tắt):
+AI so sánh Sequence Diagram của em với phiên bản đề xuất, đánh giá 8.5 – 9.0/10. Điểm mạnh: rất chi tiết, có đầy đủ participant, tách biệt BookingService &amp; PaymentService, sử dụng alt fragment và combined fragment rõ ràng. Điểm yếu: hơi nhiều lifeline khiến diagram hơi dày.
+Quyết định của người học:
+ tinh chỉnh nhẹ Sequence Diagram (giảm bớt một số return message không cần thiết và giữ cấu trúc hiện tại). Sử dụng phiên bản diagram đã vẽ để nộp bài vì đã đạt yêu cầu tốt.</t>
+  </si>
+  <si>
+    <t>dựa vào hình ảnh sequenceDiagram tôi vẽ cho bài 2 bạn hãy so sánh với Sequence Diagram do tôi tự thiết kế và Sequence Diagram do bạn đề xuất cho hệ thống AutoGo car rental.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiết kế Sequence Diagram và so sánh thiết kế của AI </t>
+  </si>
+  <si>
+    <t>Activity Diagram của bạn: 6.0 – 6.5/10
+Activity Diagram tôi đề xuất: 8.5/10
+Ưu điểm: Luồng logic cơ bản ổn, dễ hiểu.
+Nhược điểm chính: Thiếu swimlanes (yêu cầu bắt buộc), chưa thể hiện rõ trách nhiệm giữa Staff và System.
+ Điểm mạnh: luồng logic chính đúng, có decision node rõ ràng. Điểm yếu lớn: chưa có swimlanes (Staff &amp; System) – yêu cầu quan trọng của Level 2 Design.
+Quyết định của người học:
+Để tôi chỉnh sửa bằng cách thêm 2 swimlanes (Staff và System), phân chia hoạt động rõ ràng hơn và giữ lại luồng hiện tại. Sử dụng phiên bản đã chỉnh sửa để xem thế nào.</t>
+  </si>
+  <si>
+    <t>tương tự như với 2 bài lần trước thì bạn xem cái activity diagram của tôi với bạn ra sao</t>
+  </si>
+  <si>
+    <t>So sánh activity diagram</t>
+  </si>
+  <si>
+    <t>bây giờ hãy cho tôi 2 sơ đồ chuẩn hơn cho sơ đồ 1 và 2 và so sánh tại sao và chỗ nào tôi cần sửa chính xác để chuẩn hơn và sẽ tiếp cận được điểm cao hơn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check lỗi và lấy lỗi cụ thể từ AI để so sánh và chỉnh sửa </t>
+  </si>
+  <si>
+    <t>Class Diagram
+Điểm yếu hiện tại của bạn:
+Thiếu BookingService (rất quan trọng)
+Dùng Vehicle thay vì Car
+Mối quan hệ Booking-Vehicle dùng composition (black diamond) → sai
+Chưa thể hiện rõ dependency Service → Repository
+PaymentService làm quá nhiều việc
+Cần sửa:
+Thêm lớp BookingService
+Đổi Vehicle → Car
+Sửa mối quan hệ Booking-Car thành Association (mũi tên thường) 1..1
+Thêm dependency (mũi tên đứt) từ Service xuống Repository
+Tách rõ trách nhiệm giữa BookingService và PaymentService
+Sequence Diagram
+Điểm yếu hiện tại của bạn:
+Quá nhiều participant → diagram hơi rối và dày
+Một số message dài dòng, return message thừa
+Combined fragment màu vàng hơi nặng
+Cần sửa:
+Giảm bớt participant (gộp một số nếu cần)
+Rút gọn một số return message
+Giữ cấu trúc alt fragment rõ ràng như phiên bản tôi đưa
+Đảm bảo luồng BookingService → PaymentService rõ ràng</t>
   </si>
 </sst>
 </file>
@@ -859,9 +929,88 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="20.9375" style="9" customWidth="1"/>
+    <col min="2" max="2" width="60.75" style="9" customWidth="1"/>
+    <col min="3" max="3" width="39.5" style="9" customWidth="1"/>
+    <col min="4" max="4" width="52.6875" style="9" customWidth="1"/>
+    <col min="5" max="16384" width="9" style="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="13.9" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="148.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="135" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="162" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add week6 AI audit log file
</commit_message>
<xml_diff>
--- a/AI Audit Log_TRanVanDong_DE180115.xlsx
+++ b/AI Audit Log_TRanVanDong_DE180115.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Audit_log\ai-audit-log-donghocgithub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB173833-B8FA-4B66-9B7C-E452AA80AFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21CC0730-6A8D-4A61-B57C-A6C3653D902E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="5" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week1" sheetId="1" r:id="rId1"/>
     <sheet name="Week2" sheetId="2" r:id="rId2"/>
     <sheet name="Week3" sheetId="3" r:id="rId3"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Week4" sheetId="4" r:id="rId4"/>
+    <sheet name="Week5" sheetId="5" r:id="rId5"/>
+    <sheet name="Week6" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="80">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -304,6 +306,140 @@
 Rút gọn một số return message
 Giữ cấu trúc alt fragment rõ ràng như phiên bản tôi đưa
 Đảm bảo luồng BookingService → PaymentService rõ ràng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dựa vào đề của tôi bài 3 hãy vẽ cho tôi một cái luồng chuẩn chỉ cho cái state Diagram này </t>
+  </si>
+  <si>
+    <t>Phân tích và thiết kế State Diagram</t>
+  </si>
+  <si>
+    <t>Created (Khởi tạo): Khách hàng chọn món xong và bấm đặt hàng. $\rightarrow$ Sự kiện tiếp theo: Nhân viên bấm xác nhận (confirmOrder).
+Confirmed (Đã xác nhận): Đơn hàng được nhân viên tiếp nhận và hệ thống yêu cầu thanh toán. $\rightarrow$ Sự kiện tiếp theo: Khách quẹt thẻ/trả tiền mặt thành công (paySuccess).
+Paid (Đã thanh toán): Tiền đã vào hệ thống, đơn hàng hợp lệ để bắt đầu làm món. $\rightarrow$ Sự kiện tiếp theo: Bếp nhận đơn và bắt đầu nấu (startCooking).
+Preparing (Đang chuẩn bị): Đầu bếp đang xào nấu thức ăn trong bếp. $\rightarrow$ Sự kiện tiếp theo: Đầu bếp nấu xong, bấm chuông báo (finishCooking).
+ReadyToServe (Sẵn sàng phục vụ): Món ăn đã đặt lên quầy, chờ nhân viên bưng ra. $\rightarrow$ Sự kiện tiếp theo: Nhân viên bưng món đến bàn cho khách (serveOrder).
+Served (Đã phục vụ): Khách hàng đang thưởng thức món ăn. $\rightarrow$ Sự kiện tiếp theo: Khách ăn xong, rời đi, nhân viên dọn bàn và đóng đơn (closeOrder).
+Completed (Hoàn tất): Vòng đời của đơn hàng kết thúc trọn vẹn, dữ liệu lưu vào lịch sử doanh thu.
+Quyết định của người học:
+Sau khi đọc luồng chuẩn (Happy Path) AI cung cấp, tôi nhận thấy đề bài Câu 3 có yêu cầu thêm 'Alternative termination state' (nhánh rẽ thất bại). Quyết định: Yêu cầu AI bổ sung thêm các nhánh rẽ lỗi (Thanh toán thất bại, Hủy đơn) vào luồng chuẩn này để đáp ứng 100% barem điểm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dựa vào hình ảnh mẫu bạn hãy vẽ cho tôi dựa trên cái sơ đồ luồng mà nãy tôi đã cung cấp </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiết kế sơ đồ demo dựa mẫu có sẵn </t>
+  </si>
+  <si>
+    <t>hêm nút bắt đầu [*] và nút kết thúc [*].
+Phát triển từ "luồng chuẩn" ban đầu bằng cách rẽ 2 nhánh (Branching):
+Nhánh từ Created $\rightarrow$ Cancelled (Sự kiện: cancelOrder).
+Nhánh từ Confirmed đi qua khối lựa chọn (Choice) $\rightarrow$ áp dụng Guard Condition [success] để đi tới Paid và [failed] để đi tới PaymentFailed.
+Bổ sung thêm các Action (Hành động) đi kèm sự kiện như / printReceipt, / notifyCustomer cho giống phong cách học thuật của ảnh mẫu.
+Quyết định của người học:
+Khi tôi copy đoạn mã Mermaid của AI dán vào phần mềm vẽ/văn bản của mình, vì các cụm chữ trên mũi tên rẽ nhánh quá dài (ví dụ: [success] / printReceipt và [failed] / showError) nên hình ảnh render ra bị lỗi đè chữ lên nhau, và khối trạng thái lồng nhau khiến một nửa biểu đồ bị cắt mất. hãy sử dụng thẻ ngắt dòng &lt;br&gt; và loại bỏ các khối lồng ghép phức tạp.</t>
+  </si>
+  <si>
+    <t>Xác minh kiến thức</t>
+  </si>
+  <si>
+    <t>ôi sợ bị nhầm lẫn, biểu đồ này rốt cuộc là Sơ đồ hoạt động (Activity) hay Sơ đồ trạng thái (State Diagram)? Dấu hiệu nhận biết là gì?</t>
+  </si>
+  <si>
+    <t>Phản hồi của AI: (AI phân tích sự khác nhau: State Diagram dùng tính từ/danh từ chỉ tình trạng như Created, Paid; Activity Diagram dùng động từ chỉ hành động...).
+Quyết định của người học (Reflection): "Việc nhầm lẫn 2 loại biểu đồ này rất dễ xảy ra khi đi thi. Quyết định:  AI tổng hợp quy tắc đặt tên (Naming Convention) cho các khối trạng thái để tôi ghi nhớ và áp dụng cho các bài tập sau."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mở rộng bài làm </t>
+  </si>
+  <si>
+    <t>Dựa vào đề bài chung, bây giờ hãy giúp tôi phân tích các Entity và quan hệ để vẽ Class Diagram (Câu 1) sử dụng Repository Pattern</t>
+  </si>
+  <si>
+    <t>Phản hồi của AI: (AI phân tích kiến trúc Layered, liệt kê các class User, Customer, Menu... và quan hệ kế thừa/composition).
+Quyết định của người học (Reflection): "AI đã thiết kế kiến trúc rất tốt, nhưng tôi nhận thấy chưa rõ ràng về việc làm sao Tầng Service gọi được Interface Repository. Quyết định: Yêu cầu AI giải thích thêm về quan hệ Dependency ..&gt; giữa Service và Repository trong biểu đồ lớp."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">check lại lần cuối </t>
+  </si>
+  <si>
+    <t>Nhìn vào hình của tôi sau khi sửa đổi thì đúng như vậy chưa từ đường kẻ đến nút tròn …</t>
+  </si>
+  <si>
+    <t>rạng thái bắt đầu (Initial State): Nút tròn đen đặc đã xuất hiện ở trên cùng và trỏ chính xác vào khối khởi tạo Created.
+Trạng thái kết thúc (Final State): Cả 3 nhánh kết thúc (Completed, Cancelled, PaymentFailed) đều đã trỏ đúng về các vòng tròn có dấu chấm đen ở giữa (chuẩn UML cho Final State).
+Đường kẻ và Nhãn rẽ nhánh: Lỗi layout đè chữ đã được khắc phục hoàn toàn nhờ thẻ ngắt dòng. Các yếu tố học thuật như Điều kiện kiểm tra [success]/[failed] và Hành động /printReceipt đều được căn lề rõ ràng, trực quan. Biểu đồ này đã đạt mức độ hoàn hảo để bạn đưa vào báo cáo môn học!
+Quyết định của người học:
+oce</t>
+  </si>
+  <si>
+    <t>Nghiên cứu lý thuyết nền tảng</t>
+  </si>
+  <si>
+    <t>Tôi đang chuẩn bị vẽ Class Diagram cho hệ thống quản lý phòng khám (Clinic Management). Trước khi vẽ, hãy giải thích ngắn gọn cho tôi sự khác biệt giữa các mối quan hệ: Association, Aggregation và Composition trong UML để tôi áp dụng cho đúng</t>
+  </si>
+  <si>
+    <t>Phản hồi của AI: AI giải thích rõ ràng: Association là liên kết ngang hàng bình thường. Aggregation là quan hệ chứa đựng lỏng lẻo (Whole-Part, nhưng Part tồn tại độc lập được). Composition là chứa đựng chặt chẽ (Whole chết thì Part cũng bị hủy theo). Kèm theo đó AI đưa ra các ví dụ minh họa.
+Quyết định của người học:
+ Ghi chú lại kiến thức này. Tôi quyết định sẽ áp dụng quan hệ Composition (hình thoi đen) giữa Cuộc hẹn (Appointment) và Bệnh án (MedicalRecord), vì logic thực tế là một bệnh án không thể tự nhiên tồn tại nếu không có cuộc hẹn khám đó.</t>
+  </si>
+  <si>
+    <t>Nghiên cứu cấu trúc hệ thống</t>
+  </si>
+  <si>
+    <t>Giảng viên yêu cầu bản thiết kế phải sát với thực tế code (áp dụng Layered Architecture và DTO pattern). Vậy làm sao để thể hiện các tầng Controller, Service, Repository và DTO trên cùng một Class Diagram theo đúng chuẩn UML?</t>
+  </si>
+  <si>
+    <t>Phản hồi của AI: AI hướng dẫn sử dụng các Stereotypes (như &lt;&lt;controller&gt;&gt;, &lt;&lt;service&gt;&gt;, &lt;&lt;request&gt;&gt;) đặt trên tên Class để phân loại. Đồng thời AI nhấn mạnh phải dùng mũi tên đứt nét (Dependency ..&gt;) để chỉ sự phụ thuộc từ Controller $\rightarrow$ Service $\rightarrow$ Repository thay vì dùng mũi tên liên kết thông thường.
+Quyết định của người học:
+Chuyển sang bước thực hành: Tôi sẽ bắt đầu cung cấp các yêu cầu nghiệp vụ để AI phác thảo bản nháp sơ đồ các Entity cơ bản trước tiên.</t>
+  </si>
+  <si>
+    <t>Thiết kế Kiến trúc hệ thống</t>
+  </si>
+  <si>
+    <t>Biểu đồ các thực thể đã ổn. Bây giờ hãy nâng cấp nó theo chuẩn Layered Architecture: Thêm tầng Controller (để nhận API từ Client), tầng Service (xử lý logic nghiệp vụ đặt lịch) và tầng Repository Pattern (để truy xuất Database). Gắn các Stereotype (như &lt;&lt;controller&gt;&gt;, &lt;&lt;service&gt;&gt;) cho dễ nhìn nhé</t>
+  </si>
+  <si>
+    <t>Phản hồi của AI: AI vẽ lại biểu đồ, xuất hiện thêm AppointmentController, AppointmentService và các Interface như AppointmentRepository, PatientRepository. AI dùng mũi tên Dependency (nét đứt) nối từ Controller xuống Service, và từ Service xuống Repository.
+Quyết định của người học:
+AI tách biệt dữ liệu giao tiếp bằng cách áp dụng thêm DTO (Data Transfer Object) Pattern. Đồng thời bổ sung các thực thể thanh toán, bệnh án để chốt lại sơ đồ.</t>
+  </si>
+  <si>
+    <t>Phác thảo luồng cơ bản</t>
+  </si>
+  <si>
+    <t>Tôi muốn vẽ Biểu đồ tuần tự (Sequence Diagram) cho chức năng Đăng ký tài khoản Bệnh nhân (Patient Registration). Hãy vẽ cho tôi một luồng chuẩn (Happy Path) từ lúc Khách (Guest) nhập thông tin trên React Frontend, gọi API POST xuống PatientController, Service lưu thẳng vào Database và trả kết quả thành công.</t>
+  </si>
+  <si>
+    <t>Phản hồi của AI: AI phác thảo một luồng đi thẳng một lèo không rẽ nhánh: Guest $\rightarrow$ React Frontend $\rightarrow$ PatientController $\rightarrow$ PatientService $\rightarrow$ Database (INSERT User). Trả về 201 Created.
+Quyết định của người học:
+ AI hủy bỏ luồng lưu trực tiếp này. Thay vào đó, bổ sung cơ chế xác thực OTP qua Email (sử dụng JavaMailSender) trước khi cho phép tạo tài khoản.</t>
+  </si>
+  <si>
+    <t>Tăng cường Bảo mật</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nghiên cứu cấu trúc sơ đồ </t>
+  </si>
+  <si>
+    <t>Tôi sắp phải vẽ Biểu đồ tuần tự (Sequence Diagram) cho quy trình giao tiếp giữa Frontend, Backend và Database. Trước tiên, hãy giải thích ngắn gọn cho tôi các thành phần cơ bản: Lifeline là gì? Các loại mũi tên gọi hàm (Synchronous, Asynchronous, Return) khác nhau như thế nào trong UML?</t>
+  </si>
+  <si>
+    <t>Phản hồi của AI: AI giải thích: Lifeline (Đường sinh mệnh) là trục thời gian dọc từ trên xuống đại diện cho đối tượng tham gia. Mũi tên nét liền đầu tam giác đặc (Synchronous) dùng khi gọi hàm/API và phải chờ kết quả. Mũi tên đứt nét (Return) dùng để trả về kết quả (response) sau khi xử lý xong.
+Quyết định của người học:
+ể biểu đồ chuyên nghiệp, tôi quy ước sẽ bắt buộc sử dụng mũi tên đứt nét (Return Message) kèm theo các mã HTTP Status Code (như 201 Created, 400 Bad Request) từ Controller trả ngược về Frontend sau mỗi nhịp API.</t>
+  </si>
+  <si>
+    <t>Xử lý ngoại lệ và Hoàn thiện</t>
+  </si>
+  <si>
+    <t>Luồng OTP đã ổn, nhưng để hệ thống tối ưu hơn, hãy thêm một bước kiểm tra Database (isEmailTaken) ngay khi user bấm đăng ký. Thêm một khối alt thứ hai ở đầu quy trình: Nếu [Email đã tồn tại], trả về thẳng mã lỗi 409 Conflict. Chỉ khi [Email hợp lệ] thì mới tiến hành lưu tạm (savePendingRegistration) và gọi JavaMailSender gửi OTP. Hãy cho tôi bản vẽ hoàn thiện cuối cùng.</t>
+  </si>
+  <si>
+    <t>Phản hồi của AI: AI xuất ra bản vẽ cuối cùng, phức tạp và đầy đủ chi tiết. Có sự xuất hiện của 2 khối alt lớn: Khối 1 check Email trùng, khối 2 check mã OTP. Các mã HTTP (202 Accepted, 201 Created, 400 Bad Request) được gắn đúng vào từng mũi tên trả về. (Đây chính là bức ảnh sơ đồ hoàn hảo mà bạn đang có).
+Quyết định của người học:
+ản vẽ không còn điểm trừ. Tôi chốt thiết kế Sequence Diagram tại đây và đưa vào báo cáo. Quá trình làm việc này giúp tôi rèn luyện tư duy thiết kế API an toàn và cách xử lý tuần tự nhiều lớp bảo mật trong thực tế.</t>
   </si>
 </sst>
 </file>
@@ -407,6 +543,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>27363</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2581294</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>76240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Hình ảnh 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{08011C5C-7F2E-FB75-660C-445D0F27ACDE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5123238" y="12873038"/>
+          <a:ext cx="2553931" cy="5334040"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1017,9 +1202,305 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="49.9375" customWidth="1"/>
+    <col min="3" max="3" width="51.3125" customWidth="1"/>
+    <col min="4" max="4" width="74.75" customWidth="1"/>
+    <col min="6" max="6" width="58.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="13.9" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+      <c r="F1" s="9"/>
+    </row>
+    <row r="2" spans="1:6" ht="108" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="1:6" ht="94.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+    </row>
+    <row r="4" spans="1:6" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+    </row>
+    <row r="5" spans="1:6" ht="94.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8058C741-AAD0-484C-8B2C-FB9353D1B341}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="49.9375" customWidth="1"/>
+    <col min="3" max="3" width="51.3125" customWidth="1"/>
+    <col min="4" max="4" width="74.75" customWidth="1"/>
+    <col min="6" max="6" width="58.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="13.9" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+      <c r="F1" s="9"/>
+    </row>
+    <row r="2" spans="1:6" ht="81" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="1:6" ht="94.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+    </row>
+    <row r="4" spans="1:6" ht="108" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+    </row>
+    <row r="5" spans="1:6" ht="108" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBEE460-0D4D-4624-B199-B11DFE403346}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="57.875" customWidth="1"/>
+    <col min="3" max="3" width="39.5625" customWidth="1"/>
+    <col min="4" max="4" width="64.6875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="13.9" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" ht="335.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="9"/>
+    </row>
+    <row r="3" spans="1:5" ht="201" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="9"/>
+    </row>
+    <row r="4" spans="1:5" ht="229.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="9"/>
+    </row>
+    <row r="5" spans="1:5" ht="81" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="9"/>
+    </row>
+    <row r="6" spans="1:5" ht="148.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="9"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>